<commit_message>
new version of Chapter 9
</commit_message>
<xml_diff>
--- a/model_comparison.xlsx
+++ b/model_comparison.xlsx
@@ -5,18 +5,18 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gilberto/sitsbook/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gilbertocamara/sitsbook/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B6426B7-101B-564A-80BE-97B07E205671}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63C56649-7722-E14A-81D8-FCC10B584CD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="23220" windowHeight="15680" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="30540" windowHeight="18520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="rfor" sheetId="1" r:id="rId1"/>
-    <sheet name="LightTAE" sheetId="4" r:id="rId2"/>
-    <sheet name="xgboost" sheetId="2" r:id="rId3"/>
-    <sheet name="TempCNN" sheetId="3" r:id="rId4"/>
+    <sheet name="xgboost" sheetId="2" r:id="rId2"/>
+    <sheet name="TempCNN" sheetId="3" r:id="rId3"/>
+    <sheet name="LightTAE" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
@@ -84,7 +84,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="0.000"/>
+    <numFmt numFmtId="168" formatCode="0.000"/>
   </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
@@ -117,7 +117,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -416,9 +416,6 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K22"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="15.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
@@ -460,25 +457,25 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>1446</v>
+        <v>899</v>
       </c>
       <c r="C2">
         <v>2</v>
       </c>
       <c r="D2">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E2">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="F2">
-        <v>58</v>
+        <v>36</v>
       </c>
       <c r="G2">
-        <v>49</v>
+        <v>28</v>
       </c>
       <c r="H2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I2">
         <v>0</v>
@@ -487,7 +484,7 @@
         <v>0</v>
       </c>
       <c r="K2">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.2">
@@ -498,31 +495,31 @@
         <v>4</v>
       </c>
       <c r="C3">
-        <v>1442</v>
+        <v>785</v>
       </c>
       <c r="D3">
-        <v>134</v>
+        <v>72</v>
       </c>
       <c r="E3">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="F3">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="G3">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="H3">
         <v>0</v>
       </c>
       <c r="I3">
-        <v>28</v>
+        <v>4</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>115</v>
+        <v>38</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.2">
@@ -530,34 +527,34 @@
         <v>3</v>
       </c>
       <c r="B4">
+        <v>7</v>
+      </c>
+      <c r="C4">
+        <v>48</v>
+      </c>
+      <c r="D4">
+        <v>738</v>
+      </c>
+      <c r="E4">
+        <v>84</v>
+      </c>
+      <c r="F4">
+        <v>50</v>
+      </c>
+      <c r="G4">
         <v>12</v>
       </c>
-      <c r="C4">
-        <v>91</v>
-      </c>
-      <c r="D4">
-        <v>1096</v>
-      </c>
-      <c r="E4">
-        <v>138</v>
-      </c>
-      <c r="F4">
-        <v>92</v>
-      </c>
-      <c r="G4">
-        <v>27</v>
-      </c>
       <c r="H4">
         <v>0</v>
       </c>
       <c r="I4">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>62</v>
+        <v>47</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.2">
@@ -565,25 +562,25 @@
         <v>4</v>
       </c>
       <c r="B5">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="C5">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D5">
-        <v>238</v>
+        <v>113</v>
       </c>
       <c r="E5">
-        <v>1353</v>
+        <v>836</v>
       </c>
       <c r="F5">
-        <v>89</v>
+        <v>44</v>
       </c>
       <c r="G5">
         <v>16</v>
       </c>
       <c r="H5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I5">
         <v>0</v>
@@ -592,7 +589,7 @@
         <v>0</v>
       </c>
       <c r="K5">
-        <v>19</v>
+        <v>24</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.2">
@@ -600,34 +597,34 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>61</v>
+        <v>45</v>
       </c>
       <c r="C6">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="D6">
-        <v>91</v>
+        <v>52</v>
       </c>
       <c r="E6">
-        <v>72</v>
+        <v>42</v>
       </c>
       <c r="F6">
-        <v>1308</v>
+        <v>792</v>
       </c>
       <c r="G6">
-        <v>30</v>
+        <v>17</v>
       </c>
       <c r="H6">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I6">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.2">
@@ -635,22 +632,22 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>49</v>
+        <v>27</v>
       </c>
       <c r="C7">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D7">
-        <v>24</v>
+        <v>7</v>
       </c>
       <c r="E7">
-        <v>17</v>
+        <v>5</v>
       </c>
       <c r="F7">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="G7">
-        <v>1412</v>
+        <v>866</v>
       </c>
       <c r="H7">
         <v>0</v>
@@ -662,7 +659,7 @@
         <v>0</v>
       </c>
       <c r="K7">
-        <v>26</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.2">
@@ -670,13 +667,13 @@
         <v>7</v>
       </c>
       <c r="B8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C8">
         <v>0</v>
       </c>
       <c r="D8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E8">
         <v>0</v>
@@ -688,13 +685,13 @@
         <v>0</v>
       </c>
       <c r="H8">
-        <v>496</v>
+        <v>500</v>
       </c>
       <c r="I8">
         <v>0</v>
       </c>
       <c r="J8">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K8">
         <v>0</v>
@@ -705,34 +702,34 @@
         <v>8</v>
       </c>
       <c r="B9">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C9">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="D9">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="E9">
         <v>0</v>
       </c>
       <c r="F9">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="G9">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H9">
         <v>0</v>
       </c>
       <c r="I9">
-        <v>448</v>
+        <v>492</v>
       </c>
       <c r="J9">
         <v>0</v>
       </c>
       <c r="K9">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.2">
@@ -743,13 +740,13 @@
         <v>0</v>
       </c>
       <c r="C10">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D10">
         <v>0</v>
       </c>
       <c r="E10">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F10">
         <v>0</v>
@@ -764,7 +761,7 @@
         <v>0</v>
       </c>
       <c r="J10">
-        <v>494</v>
+        <v>500</v>
       </c>
       <c r="K10">
         <v>0</v>
@@ -775,10 +772,10 @@
         <v>10</v>
       </c>
       <c r="B11">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="C11">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D11">
         <v>3</v>
@@ -790,19 +787,19 @@
         <v>3</v>
       </c>
       <c r="G11">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H11">
         <v>0</v>
       </c>
       <c r="I11">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="J11">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K11">
-        <v>562</v>
+        <v>668</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.2">
@@ -817,16 +814,16 @@
       <c r="A14" t="s">
         <v>12</v>
       </c>
-      <c r="B14">
-        <v>0.85048625792811805</v>
+      <c r="B14" s="1">
+        <v>0.879115418064356</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>13</v>
       </c>
-      <c r="B15">
-        <v>0.83023644041318201</v>
+      <c r="B15" s="1">
+        <v>0.86466693447544496</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.2">
@@ -869,34 +866,34 @@
         <v>14</v>
       </c>
       <c r="B19" s="1">
-        <v>0.90375000000000005</v>
+        <v>0.90261044176706795</v>
       </c>
       <c r="C19" s="1">
-        <v>0.91265822784810102</v>
+        <v>0.90022935779816504</v>
       </c>
       <c r="D19" s="1">
-        <v>0.68500000000000005</v>
+        <v>0.74395161290322598</v>
       </c>
       <c r="E19" s="1">
-        <v>0.84987437185929604</v>
+        <v>0.85306122448979604</v>
       </c>
       <c r="F19" s="1">
-        <v>0.8175</v>
+        <v>0.82499999999999996</v>
       </c>
       <c r="G19" s="1">
-        <v>0.91214470284237703</v>
+        <v>0.91737288135593198</v>
       </c>
       <c r="H19" s="1">
-        <v>0.99199999999999999</v>
+        <v>1</v>
       </c>
       <c r="I19" s="1">
-        <v>0.89600000000000002</v>
+        <v>0.98399999999999999</v>
       </c>
       <c r="J19" s="1">
-        <v>0.98799999999999999</v>
+        <v>1</v>
       </c>
       <c r="K19" s="1">
-        <v>0.69813664596273295</v>
+        <v>0.82981366459627304</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.2">
@@ -904,34 +901,34 @@
         <v>15</v>
       </c>
       <c r="B20" s="1">
-        <v>0.98777506112469404</v>
+        <v>0.98837374167021097</v>
       </c>
       <c r="C20" s="1">
-        <v>0.96993655441678905</v>
+        <v>0.98174724815382497</v>
       </c>
       <c r="D20" s="1">
-        <v>0.95804400977995097</v>
+        <v>0.96471588493694205</v>
       </c>
       <c r="E20" s="1">
-        <v>0.96237662464575402</v>
+        <v>0.96958551421700401</v>
       </c>
       <c r="F20" s="1">
-        <v>0.97183374083129603</v>
+        <v>0.97587812103258598</v>
       </c>
       <c r="G20" s="1">
-        <v>0.98569621484869097</v>
+        <v>0.98888106966924705</v>
       </c>
       <c r="H20" s="1">
-        <v>0.99929359823399599</v>
+        <v>0.99986753212346002</v>
       </c>
       <c r="I20" s="1">
-        <v>0.99673289183223002</v>
+        <v>0.99801298185190102</v>
       </c>
       <c r="J20" s="1">
-        <v>1</v>
+        <v>0.99973506424692005</v>
       </c>
       <c r="K20" s="1">
-        <v>0.99627949183303099</v>
+        <v>0.99613473219215898</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.2">
@@ -939,34 +936,34 @@
         <v>16</v>
       </c>
       <c r="B21" s="1">
-        <v>0.92043284532145098</v>
+        <v>0.91641182466870597</v>
       </c>
       <c r="C21" s="1">
-        <v>0.82399999999999995</v>
+        <v>0.85698689956331897</v>
       </c>
       <c r="D21" s="1">
-        <v>0.71868852459016397</v>
+        <v>0.74772036474164105</v>
       </c>
       <c r="E21" s="1">
-        <v>0.778481012658228</v>
+        <v>0.795432921027593</v>
       </c>
       <c r="F21" s="1">
-        <v>0.81954887218045103</v>
+        <v>0.82242990654205606</v>
       </c>
       <c r="G21" s="1">
-        <v>0.90570878768441299</v>
+        <v>0.916402116402117</v>
       </c>
       <c r="H21" s="1">
-        <v>0.98412698412698296</v>
+        <v>0.99800399201596701</v>
       </c>
       <c r="I21" s="1">
-        <v>0.92371134020618495</v>
+        <v>0.97041420118343202</v>
       </c>
       <c r="J21" s="1">
-        <v>1</v>
+        <v>0.99601593625498097</v>
       </c>
       <c r="K21" s="1">
-        <v>0.93200663349917101</v>
+        <v>0.95977011494252795</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.2">
@@ -974,34 +971,34 @@
         <v>17</v>
       </c>
       <c r="B22" s="1">
-        <v>0.98498147064560204</v>
+        <v>0.98627617430673498</v>
       </c>
       <c r="C22" s="1">
-        <v>0.98630272952853604</v>
+        <v>0.98780316837235405</v>
       </c>
       <c r="D22" s="1">
-        <v>0.95106796116504899</v>
+        <v>0.964032851883319</v>
       </c>
       <c r="E22" s="1">
-        <v>0.97630613661148002</v>
+        <v>0.97942269219777101</v>
       </c>
       <c r="F22" s="1">
-        <v>0.97145371004008196</v>
+        <v>0.976291278577477</v>
       </c>
       <c r="G22" s="1">
-        <v>0.98675238651860497</v>
+        <v>0.98902027027026995</v>
       </c>
       <c r="H22" s="1">
-        <v>0.99964667432205601</v>
+        <v>1</v>
       </c>
       <c r="I22" s="1">
-        <v>0.99541446208112905</v>
+        <v>0.99893927340228095</v>
       </c>
       <c r="J22" s="1">
-        <v>0.99947047921630905</v>
+        <v>1</v>
       </c>
       <c r="K22" s="1">
-        <v>0.97834610586348203</v>
+        <v>0.98136814905480796</v>
       </c>
     </row>
   </sheetData>
@@ -1011,12 +1008,9 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:K22"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="16.33203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
@@ -1058,22 +1052,22 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>1424</v>
+        <v>887</v>
       </c>
       <c r="C2">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D2">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E2">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="F2">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="G2">
-        <v>49</v>
+        <v>23</v>
       </c>
       <c r="H2">
         <v>0</v>
@@ -1085,7 +1079,7 @@
         <v>0</v>
       </c>
       <c r="K2">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.2">
@@ -1093,22 +1087,22 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C3">
-        <v>1380</v>
+        <v>779</v>
       </c>
       <c r="D3">
-        <v>136</v>
+        <v>67</v>
       </c>
       <c r="E3">
         <v>4</v>
       </c>
       <c r="F3">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="G3">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H3">
         <v>0</v>
@@ -1120,7 +1114,7 @@
         <v>0</v>
       </c>
       <c r="K3">
-        <v>105</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.2">
@@ -1128,34 +1122,34 @@
         <v>3</v>
       </c>
       <c r="B4">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C4">
-        <v>138</v>
+        <v>60</v>
       </c>
       <c r="D4">
-        <v>1104</v>
+        <v>756</v>
       </c>
       <c r="E4">
-        <v>170</v>
+        <v>84</v>
       </c>
       <c r="F4">
-        <v>89</v>
+        <v>43</v>
       </c>
       <c r="G4">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H4">
         <v>0</v>
       </c>
       <c r="I4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K4">
-        <v>44</v>
+        <v>37</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.2">
@@ -1163,25 +1157,25 @@
         <v>4</v>
       </c>
       <c r="B5">
-        <v>19</v>
+        <v>7</v>
       </c>
       <c r="C5">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D5">
-        <v>266</v>
+        <v>111</v>
       </c>
       <c r="E5">
-        <v>1353</v>
+        <v>853</v>
       </c>
       <c r="F5">
-        <v>129</v>
+        <v>48</v>
       </c>
       <c r="G5">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="H5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I5">
         <v>0</v>
@@ -1198,34 +1192,34 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>80</v>
+        <v>57</v>
       </c>
       <c r="C6">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="D6">
-        <v>70</v>
+        <v>37</v>
       </c>
       <c r="E6">
-        <v>51</v>
+        <v>24</v>
       </c>
       <c r="F6">
-        <v>1304</v>
+        <v>815</v>
       </c>
       <c r="G6">
-        <v>43</v>
+        <v>14</v>
       </c>
       <c r="H6">
         <v>0</v>
       </c>
       <c r="I6">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.2">
@@ -1233,10 +1227,10 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>54</v>
+        <v>32</v>
       </c>
       <c r="C7">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D7">
         <v>7</v>
@@ -1245,10 +1239,10 @@
         <v>5</v>
       </c>
       <c r="F7">
-        <v>23</v>
+        <v>9</v>
       </c>
       <c r="G7">
-        <v>1414</v>
+        <v>882</v>
       </c>
       <c r="H7">
         <v>0</v>
@@ -1260,7 +1254,7 @@
         <v>0</v>
       </c>
       <c r="K7">
-        <v>16</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.2">
@@ -1268,31 +1262,31 @@
         <v>7</v>
       </c>
       <c r="B8">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C8">
         <v>0</v>
       </c>
       <c r="D8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G8">
         <v>0</v>
       </c>
       <c r="H8">
-        <v>496</v>
+        <v>500</v>
       </c>
       <c r="I8">
         <v>0</v>
       </c>
       <c r="J8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K8">
         <v>0</v>
@@ -1303,28 +1297,28 @@
         <v>8</v>
       </c>
       <c r="B9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C9">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H9">
         <v>0</v>
       </c>
       <c r="I9">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="J9">
         <v>0</v>
@@ -1341,10 +1335,10 @@
         <v>0</v>
       </c>
       <c r="C10">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D10">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E10">
         <v>1</v>
@@ -1356,7 +1350,7 @@
         <v>0</v>
       </c>
       <c r="H10">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I10">
         <v>0</v>
@@ -1373,34 +1367,34 @@
         <v>10</v>
       </c>
       <c r="B11">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="C11">
-        <v>23</v>
+        <v>11</v>
       </c>
       <c r="D11">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="E11">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F11">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H11">
         <v>0</v>
       </c>
       <c r="I11">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J11">
         <v>0</v>
       </c>
       <c r="K11">
-        <v>593</v>
+        <v>699</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.2">
@@ -1415,16 +1409,16 @@
       <c r="A14" t="s">
         <v>12</v>
       </c>
-      <c r="B14">
-        <v>0.85006342494714604</v>
+      <c r="B14" s="1">
+        <v>0.88905454093676195</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>13</v>
       </c>
-      <c r="B15">
-        <v>0.829814558832209</v>
+      <c r="B15" s="1">
+        <v>0.87578494197156498</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.2">
@@ -1467,34 +1461,34 @@
         <v>14</v>
       </c>
       <c r="B19" s="1">
-        <v>0.89</v>
+        <v>0.89056224899598402</v>
       </c>
       <c r="C19" s="1">
-        <v>0.873417721518987</v>
+        <v>0.89334862385321101</v>
       </c>
       <c r="D19" s="1">
-        <v>0.69</v>
+        <v>0.76209677419354804</v>
       </c>
       <c r="E19" s="1">
-        <v>0.84987437185929604</v>
+        <v>0.87040816326530601</v>
       </c>
       <c r="F19" s="1">
-        <v>0.81499999999999995</v>
+        <v>0.84895833333333304</v>
       </c>
       <c r="G19" s="1">
-        <v>0.91343669250645998</v>
+        <v>0.93432203389830504</v>
       </c>
       <c r="H19" s="1">
-        <v>0.99199999999999999</v>
+        <v>1</v>
       </c>
       <c r="I19" s="1">
-        <v>0.97</v>
+        <v>0.97199999999999998</v>
       </c>
       <c r="J19" s="1">
         <v>0.998</v>
       </c>
       <c r="K19" s="1">
-        <v>0.73664596273291905</v>
+        <v>0.86832298136646002</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.2">
@@ -1502,34 +1496,34 @@
         <v>15</v>
       </c>
       <c r="B20" s="1">
-        <v>0.98806845965770196</v>
+        <v>0.98851552530837905</v>
       </c>
       <c r="C20" s="1">
-        <v>0.97452415812591497</v>
+        <v>0.98592726766058203</v>
       </c>
       <c r="D20" s="1">
-        <v>0.95481662591687</v>
+        <v>0.96542440130367002</v>
       </c>
       <c r="E20" s="1">
-        <v>0.95377699599335497</v>
+        <v>0.97015136511529199</v>
       </c>
       <c r="F20" s="1">
-        <v>0.97251833740831295</v>
+        <v>0.97884045704612799</v>
       </c>
       <c r="G20" s="1">
-        <v>0.98929648730174202</v>
+        <v>0.99099225897255405</v>
       </c>
       <c r="H20" s="1">
-        <v>0.99947019867549702</v>
+        <v>0.99986753212346002</v>
       </c>
       <c r="I20" s="1">
-        <v>0.99947019867549702</v>
+        <v>0.99867532123460101</v>
       </c>
       <c r="J20" s="1">
-        <v>0.99938189845474601</v>
+        <v>0.99986753212346002</v>
       </c>
       <c r="K20" s="1">
-        <v>0.99591651542649695</v>
+        <v>0.99585864163445603</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.2">
@@ -1537,34 +1531,34 @@
         <v>16</v>
       </c>
       <c r="B21" s="1">
-        <v>0.92108667529107402</v>
+        <v>0.91632231404958697</v>
       </c>
       <c r="C21" s="1">
-        <v>0.84095063985374796</v>
+        <v>0.88522727272727197</v>
       </c>
       <c r="D21" s="1">
-        <v>0.70498084291187801</v>
+        <v>0.75600000000000001</v>
       </c>
       <c r="E21" s="1">
-        <v>0.74096385542168697</v>
+        <v>0.80169172932330801</v>
       </c>
       <c r="F21" s="1">
-        <v>0.82271293375394305</v>
+        <v>0.84455958549222798</v>
       </c>
       <c r="G21" s="1">
-        <v>0.92782152230971204</v>
+        <v>0.93234672304439703</v>
       </c>
       <c r="H21" s="1">
-        <v>0.98804780876494003</v>
+        <v>0.99800399201596701</v>
       </c>
       <c r="I21" s="1">
-        <v>0.98778004073319803</v>
+        <v>0.97983870967741904</v>
       </c>
       <c r="J21" s="1">
-        <v>0.98616600790513798</v>
+        <v>0.997999999999999</v>
       </c>
       <c r="K21" s="1">
-        <v>0.92946708463949901</v>
+        <v>0.95884773662551503</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.2">
@@ -1572,34 +1566,34 @@
         <v>17</v>
       </c>
       <c r="B22" s="1">
-        <v>0.98287771183967299</v>
+        <v>0.98460669396977796</v>
       </c>
       <c r="C22" s="1">
-        <v>0.98036135113904199</v>
+        <v>0.987027479425303</v>
       </c>
       <c r="D22" s="1">
-        <v>0.95165220781752602</v>
+        <v>0.96652007376932902</v>
       </c>
       <c r="E22" s="1">
-        <v>0.97609760976097604</v>
+        <v>0.98181818181818203</v>
       </c>
       <c r="F22" s="1">
-        <v>0.97109374999999998</v>
+        <v>0.97953133822699001</v>
       </c>
       <c r="G22" s="1">
-        <v>0.98699155421803697</v>
+        <v>0.99127129381951296</v>
       </c>
       <c r="H22" s="1">
-        <v>0.99964673673054805</v>
+        <v>1</v>
       </c>
       <c r="I22" s="1">
-        <v>0.99867654843832698</v>
+        <v>0.99814643188137198</v>
       </c>
       <c r="J22" s="1">
-        <v>0.99991165297287699</v>
+        <v>0.99986753212346002</v>
       </c>
       <c r="K22" s="1">
-        <v>0.98104943237686604</v>
+        <v>0.98551912568305999</v>
       </c>
     </row>
   </sheetData>
@@ -1609,7 +1603,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:K22"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
@@ -1653,22 +1647,22 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>1446</v>
+        <v>898</v>
       </c>
       <c r="C2">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E2">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="F2">
-        <v>45</v>
+        <v>23</v>
       </c>
       <c r="G2">
-        <v>37</v>
+        <v>17</v>
       </c>
       <c r="H2">
         <v>0</v>
@@ -1680,7 +1674,7 @@
         <v>0</v>
       </c>
       <c r="K2">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.2">
@@ -1688,34 +1682,34 @@
         <v>2</v>
       </c>
       <c r="B3">
+        <v>4</v>
+      </c>
+      <c r="C3">
+        <v>772</v>
+      </c>
+      <c r="D3">
+        <v>85</v>
+      </c>
+      <c r="E3">
         <v>5</v>
       </c>
-      <c r="C3">
-        <v>1416</v>
-      </c>
-      <c r="D3">
-        <v>121</v>
-      </c>
-      <c r="E3">
-        <v>7</v>
-      </c>
       <c r="F3">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G3">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="H3">
         <v>0</v>
       </c>
       <c r="I3">
-        <v>23</v>
+        <v>2</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>100</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.2">
@@ -1723,34 +1717,34 @@
         <v>3</v>
       </c>
       <c r="B4">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="C4">
-        <v>119</v>
+        <v>73</v>
       </c>
       <c r="D4">
-        <v>1126</v>
+        <v>738</v>
       </c>
       <c r="E4">
-        <v>150</v>
+        <v>88</v>
       </c>
       <c r="F4">
-        <v>90</v>
+        <v>39</v>
       </c>
       <c r="G4">
-        <v>30</v>
+        <v>2</v>
       </c>
       <c r="H4">
         <v>0</v>
       </c>
       <c r="I4">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>60</v>
+        <v>18</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.2">
@@ -1758,22 +1752,22 @@
         <v>4</v>
       </c>
       <c r="B5">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="C5">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="D5">
-        <v>234</v>
+        <v>116</v>
       </c>
       <c r="E5">
-        <v>1345</v>
+        <v>849</v>
       </c>
       <c r="F5">
-        <v>94</v>
+        <v>51</v>
       </c>
       <c r="G5">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="H5">
         <v>0</v>
@@ -1785,7 +1779,7 @@
         <v>0</v>
       </c>
       <c r="K5">
-        <v>18</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.2">
@@ -1793,34 +1787,34 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>70</v>
+        <v>47</v>
       </c>
       <c r="C6">
         <v>5</v>
       </c>
       <c r="D6">
-        <v>88</v>
+        <v>38</v>
       </c>
       <c r="E6">
-        <v>66</v>
+        <v>29</v>
       </c>
       <c r="F6">
-        <v>1325</v>
+        <v>823</v>
       </c>
       <c r="G6">
-        <v>49</v>
+        <v>14</v>
       </c>
       <c r="H6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I6">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.2">
@@ -1828,34 +1822,34 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="C7">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D7">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="E7">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="F7">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="G7">
-        <v>1399</v>
+        <v>905</v>
       </c>
       <c r="H7">
         <v>0</v>
       </c>
       <c r="I7">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>20</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.2">
@@ -1863,16 +1857,16 @@
         <v>7</v>
       </c>
       <c r="B8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C8">
         <v>0</v>
       </c>
       <c r="D8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F8">
         <v>1</v>
@@ -1881,13 +1875,13 @@
         <v>0</v>
       </c>
       <c r="H8">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="I8">
         <v>0</v>
       </c>
       <c r="J8">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K8">
         <v>0</v>
@@ -1898,34 +1892,34 @@
         <v>8</v>
       </c>
       <c r="B9">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C9">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="D9">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="E9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F9">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G9">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H9">
         <v>0</v>
       </c>
       <c r="I9">
-        <v>449</v>
+        <v>493</v>
       </c>
       <c r="J9">
         <v>0</v>
       </c>
       <c r="K9">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.2">
@@ -1942,7 +1936,7 @@
         <v>0</v>
       </c>
       <c r="E10">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F10">
         <v>0</v>
@@ -1957,7 +1951,7 @@
         <v>0</v>
       </c>
       <c r="J10">
-        <v>497</v>
+        <v>500</v>
       </c>
       <c r="K10">
         <v>0</v>
@@ -1968,34 +1962,34 @@
         <v>10</v>
       </c>
       <c r="B11">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="C11">
-        <v>23</v>
+        <v>7</v>
       </c>
       <c r="D11">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E11">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F11">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="G11">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="H11">
         <v>0</v>
       </c>
       <c r="I11">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="J11">
         <v>0</v>
       </c>
       <c r="K11">
-        <v>587</v>
+        <v>744</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.2">
@@ -2010,16 +2004,16 @@
       <c r="A14" t="s">
         <v>12</v>
       </c>
-      <c r="B14">
-        <v>0.85319238900634298</v>
+      <c r="B14" s="1">
+        <v>0.89725431730649796</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>13</v>
       </c>
-      <c r="B15">
-        <v>0.83334979821502098</v>
+      <c r="B15" s="1">
+        <v>0.88498567418714802</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.2">
@@ -2061,140 +2055,140 @@
       <c r="A19" t="s">
         <v>14</v>
       </c>
-      <c r="B19">
-        <v>0.90375000000000005</v>
-      </c>
-      <c r="C19">
-        <v>0.89620253164556996</v>
-      </c>
-      <c r="D19">
-        <v>0.70374999999999999</v>
-      </c>
-      <c r="E19">
-        <v>0.84484924623115598</v>
-      </c>
-      <c r="F19">
-        <v>0.828125</v>
-      </c>
-      <c r="G19">
-        <v>0.90374677002584003</v>
-      </c>
-      <c r="H19">
-        <v>0.998</v>
-      </c>
-      <c r="I19">
-        <v>0.89800000000000002</v>
-      </c>
-      <c r="J19">
-        <v>0.99399999999999999</v>
-      </c>
-      <c r="K19">
-        <v>0.72919254658385102</v>
+      <c r="B19" s="1">
+        <v>0.90160642570281102</v>
+      </c>
+      <c r="C19" s="1">
+        <v>0.88532110091743099</v>
+      </c>
+      <c r="D19" s="1">
+        <v>0.74395161290322598</v>
+      </c>
+      <c r="E19" s="1">
+        <v>0.86632653061224496</v>
+      </c>
+      <c r="F19" s="1">
+        <v>0.85729166666666701</v>
+      </c>
+      <c r="G19" s="1">
+        <v>0.95868644067796605</v>
+      </c>
+      <c r="H19" s="1">
+        <v>1</v>
+      </c>
+      <c r="I19" s="1">
+        <v>0.98599999999999999</v>
+      </c>
+      <c r="J19" s="1">
+        <v>1</v>
+      </c>
+      <c r="K19" s="1">
+        <v>0.924223602484472</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>15</v>
       </c>
-      <c r="B20">
-        <v>0.99012224938875304</v>
-      </c>
-      <c r="C20">
-        <v>0.97345046364080001</v>
-      </c>
-      <c r="D20">
-        <v>0.95432762836185803</v>
-      </c>
-      <c r="E20">
-        <v>0.96257207075148998</v>
-      </c>
-      <c r="F20">
-        <v>0.97056234718826395</v>
-      </c>
-      <c r="G20">
-        <v>0.98871265933638197</v>
-      </c>
-      <c r="H20">
-        <v>0.99947019867549702</v>
-      </c>
-      <c r="I20">
-        <v>0.99717439293598198</v>
-      </c>
-      <c r="J20">
-        <v>0.99991169977924899</v>
-      </c>
-      <c r="K20">
-        <v>0.99482758620689704</v>
+      <c r="B20" s="1">
+        <v>0.99291081809159198</v>
+      </c>
+      <c r="C20" s="1">
+        <v>0.98369792392364497</v>
+      </c>
+      <c r="D20" s="1">
+        <v>0.96797506022389102</v>
+      </c>
+      <c r="E20" s="1">
+        <v>0.97213184325930102</v>
+      </c>
+      <c r="F20" s="1">
+        <v>0.97968683876428297</v>
+      </c>
+      <c r="G20" s="1">
+        <v>0.99127375087966196</v>
+      </c>
+      <c r="H20" s="1">
+        <v>0.99973506424692005</v>
+      </c>
+      <c r="I20" s="1">
+        <v>0.99960259637037996</v>
+      </c>
+      <c r="J20" s="1">
+        <v>1</v>
+      </c>
+      <c r="K20" s="1">
+        <v>0.99641082274986204</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>16</v>
       </c>
-      <c r="B21">
-        <v>0.93471234647705204</v>
-      </c>
-      <c r="C21">
-        <v>0.83886255924170605</v>
-      </c>
-      <c r="D21">
-        <v>0.70684243565599503</v>
-      </c>
-      <c r="E21">
-        <v>0.77835648148148195</v>
-      </c>
-      <c r="F21">
-        <v>0.81488314883148805</v>
-      </c>
-      <c r="G21">
-        <v>0.92343234323432299</v>
-      </c>
-      <c r="H21">
-        <v>0.988118811881188</v>
-      </c>
-      <c r="I21">
-        <v>0.93347193347193302</v>
-      </c>
-      <c r="J21">
-        <v>0.99799196787148603</v>
-      </c>
-      <c r="K21">
-        <v>0.91149068322981397</v>
+      <c r="B21" s="1">
+        <v>0.94725738396624504</v>
+      </c>
+      <c r="C21" s="1">
+        <v>0.86839145106861604</v>
+      </c>
+      <c r="D21" s="1">
+        <v>0.76556016597510301</v>
+      </c>
+      <c r="E21" s="1">
+        <v>0.81166347992351795</v>
+      </c>
+      <c r="F21" s="1">
+        <v>0.851085832471561</v>
+      </c>
+      <c r="G21" s="1">
+        <v>0.93588417786970002</v>
+      </c>
+      <c r="H21" s="1">
+        <v>0.99601593625498097</v>
+      </c>
+      <c r="I21" s="1">
+        <v>0.99395161290322598</v>
+      </c>
+      <c r="J21" s="1">
+        <v>1</v>
+      </c>
+      <c r="K21" s="1">
+        <v>0.966233766233766</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>17</v>
       </c>
-      <c r="B22">
-        <v>0.98501654018291496</v>
-      </c>
-      <c r="C22">
-        <v>0.98382164348426604</v>
-      </c>
-      <c r="D22">
-        <v>0.95367474589523105</v>
-      </c>
-      <c r="E22">
-        <v>0.97553728830345598</v>
-      </c>
-      <c r="F22">
-        <v>0.97303657221296203</v>
-      </c>
-      <c r="G22">
-        <v>0.98554801163918504</v>
-      </c>
-      <c r="H22">
-        <v>0.99991166077738503</v>
-      </c>
-      <c r="I22">
-        <v>0.99550423131170696</v>
-      </c>
-      <c r="J22">
-        <v>0.99973514611106196</v>
-      </c>
-      <c r="K22">
-        <v>0.98050263840443597</v>
+      <c r="B22" s="1">
+        <v>0.98619912688353795</v>
+      </c>
+      <c r="C22" s="1">
+        <v>0.98603351955307295</v>
+      </c>
+      <c r="D22" s="1">
+        <v>0.96414961185603398</v>
+      </c>
+      <c r="E22" s="1">
+        <v>0.98129373125803199</v>
+      </c>
+      <c r="F22" s="1">
+        <v>0.98065518215193404</v>
+      </c>
+      <c r="G22" s="1">
+        <v>0.99449308105055101</v>
+      </c>
+      <c r="H22" s="1">
+        <v>1</v>
+      </c>
+      <c r="I22" s="1">
+        <v>0.99907321594068599</v>
+      </c>
+      <c r="J22" s="1">
+        <v>1</v>
+      </c>
+      <c r="K22" s="1">
+        <v>0.99161972798461295</v>
       </c>
     </row>
   </sheetData>
@@ -2204,7 +2198,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:K22"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
@@ -2248,10 +2242,10 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>1446</v>
+        <v>891</v>
       </c>
       <c r="C2">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="D2">
         <v>7</v>
@@ -2260,10 +2254,10 @@
         <v>2</v>
       </c>
       <c r="F2">
-        <v>46</v>
+        <v>30</v>
       </c>
       <c r="G2">
-        <v>47</v>
+        <v>20</v>
       </c>
       <c r="H2">
         <v>0</v>
@@ -2275,7 +2269,7 @@
         <v>0</v>
       </c>
       <c r="K2">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.2">
@@ -2283,34 +2277,34 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="C3">
-        <v>1375</v>
+        <v>777</v>
       </c>
       <c r="D3">
-        <v>140</v>
+        <v>91</v>
       </c>
       <c r="E3">
         <v>6</v>
       </c>
       <c r="F3">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="G3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H3">
         <v>0</v>
       </c>
       <c r="I3">
-        <v>53</v>
+        <v>0</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>55</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.2">
@@ -2318,34 +2312,34 @@
         <v>3</v>
       </c>
       <c r="B4">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="C4">
-        <v>118</v>
+        <v>49</v>
       </c>
       <c r="D4">
-        <v>1129</v>
+        <v>713</v>
       </c>
       <c r="E4">
-        <v>151</v>
+        <v>94</v>
       </c>
       <c r="F4">
-        <v>83</v>
+        <v>37</v>
       </c>
       <c r="G4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H4">
         <v>0</v>
       </c>
       <c r="I4">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>58</v>
+        <v>13</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.2">
@@ -2356,19 +2350,19 @@
         <v>8</v>
       </c>
       <c r="C5">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D5">
-        <v>234</v>
+        <v>121</v>
       </c>
       <c r="E5">
-        <v>1360</v>
+        <v>835</v>
       </c>
       <c r="F5">
-        <v>73</v>
+        <v>34</v>
       </c>
       <c r="G5">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="H5">
         <v>0</v>
@@ -2388,34 +2382,34 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>82</v>
+        <v>44</v>
       </c>
       <c r="C6">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="D6">
-        <v>72</v>
+        <v>35</v>
       </c>
       <c r="E6">
-        <v>59</v>
+        <v>28</v>
       </c>
       <c r="F6">
-        <v>1355</v>
+        <v>825</v>
       </c>
       <c r="G6">
-        <v>38</v>
+        <v>13</v>
       </c>
       <c r="H6">
         <v>0</v>
       </c>
       <c r="I6">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>19</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.2">
@@ -2423,34 +2417,34 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C7">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D7">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="E7">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F7">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="G7">
-        <v>1440</v>
+        <v>905</v>
       </c>
       <c r="H7">
         <v>0</v>
       </c>
       <c r="I7">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>21</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.2">
@@ -2458,31 +2452,31 @@
         <v>7</v>
       </c>
       <c r="B8">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C8">
         <v>0</v>
       </c>
       <c r="D8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G8">
         <v>0</v>
       </c>
       <c r="H8">
-        <v>498</v>
+        <v>500</v>
       </c>
       <c r="I8">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J8">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K8">
         <v>0</v>
@@ -2493,28 +2487,28 @@
         <v>8</v>
       </c>
       <c r="B9">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C9">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E9">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F9">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G9">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H9">
         <v>0</v>
       </c>
       <c r="I9">
-        <v>393</v>
+        <v>498</v>
       </c>
       <c r="J9">
         <v>0</v>
@@ -2531,10 +2525,10 @@
         <v>0</v>
       </c>
       <c r="C10">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D10">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E10">
         <v>1</v>
@@ -2546,13 +2540,13 @@
         <v>0</v>
       </c>
       <c r="H10">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I10">
         <v>0</v>
       </c>
       <c r="J10">
-        <v>497</v>
+        <v>500</v>
       </c>
       <c r="K10">
         <v>0</v>
@@ -2566,31 +2560,31 @@
         <v>4</v>
       </c>
       <c r="C11">
-        <v>44</v>
+        <v>19</v>
       </c>
       <c r="D11">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E11">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F11">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H11">
         <v>0</v>
       </c>
       <c r="I11">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="J11">
         <v>0</v>
       </c>
       <c r="K11">
-        <v>629</v>
+        <v>751</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.2">
@@ -2605,16 +2599,16 @@
       <c r="A14" t="s">
         <v>12</v>
       </c>
-      <c r="B14">
-        <v>0.85598308668076095</v>
+      <c r="B14" s="1">
+        <v>0.89389986333706095</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>13</v>
       </c>
-      <c r="B15">
-        <v>0.83650059494518003</v>
+      <c r="B15" s="1">
+        <v>0.88124949544157305</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.2">
@@ -2656,140 +2650,140 @@
       <c r="A19" t="s">
         <v>14</v>
       </c>
-      <c r="B19">
-        <v>0.90375000000000005</v>
-      </c>
-      <c r="C19">
-        <v>0.870253164556962</v>
-      </c>
-      <c r="D19">
-        <v>0.70562499999999995</v>
-      </c>
-      <c r="E19">
-        <v>0.85427135678391997</v>
-      </c>
-      <c r="F19">
-        <v>0.84687500000000004</v>
-      </c>
-      <c r="G19">
-        <v>0.93023255813953498</v>
-      </c>
-      <c r="H19">
+      <c r="B19" s="1">
+        <v>0.89457831325301196</v>
+      </c>
+      <c r="C19" s="1">
+        <v>0.89105504587156004</v>
+      </c>
+      <c r="D19" s="1">
+        <v>0.71875</v>
+      </c>
+      <c r="E19" s="1">
+        <v>0.85204081632653095</v>
+      </c>
+      <c r="F19" s="1">
+        <v>0.859375</v>
+      </c>
+      <c r="G19" s="1">
+        <v>0.95868644067796605</v>
+      </c>
+      <c r="H19" s="1">
+        <v>1</v>
+      </c>
+      <c r="I19" s="1">
         <v>0.996</v>
       </c>
-      <c r="I19">
-        <v>0.78600000000000003</v>
-      </c>
-      <c r="J19">
-        <v>0.99399999999999999</v>
-      </c>
-      <c r="K19">
-        <v>0.78136645962732898</v>
+      <c r="J19" s="1">
+        <v>1</v>
+      </c>
+      <c r="K19" s="1">
+        <v>0.93291925465838499</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>15</v>
       </c>
-      <c r="B20">
-        <v>0.98875305623471899</v>
-      </c>
-      <c r="C20">
-        <v>0.97296242069302097</v>
-      </c>
-      <c r="D20">
-        <v>0.95745721271393602</v>
-      </c>
-      <c r="E20">
-        <v>0.96530831623179902</v>
-      </c>
-      <c r="F20">
-        <v>0.97124694376528098</v>
-      </c>
-      <c r="G20">
-        <v>0.98949109662352797</v>
-      </c>
-      <c r="H20">
-        <v>0.99911699779249497</v>
-      </c>
-      <c r="I20">
-        <v>0.99858719646799099</v>
-      </c>
-      <c r="J20">
-        <v>0.99964679911699805</v>
-      </c>
-      <c r="K20">
-        <v>0.99192377495462802</v>
+      <c r="B20" s="1">
+        <v>0.99064227988090203</v>
+      </c>
+      <c r="C20" s="1">
+        <v>0.98439459384143801</v>
+      </c>
+      <c r="D20" s="1">
+        <v>0.97151764205753199</v>
+      </c>
+      <c r="E20" s="1">
+        <v>0.97312208233130604</v>
+      </c>
+      <c r="F20" s="1">
+        <v>0.98081534772182299</v>
+      </c>
+      <c r="G20" s="1">
+        <v>0.98662913441238598</v>
+      </c>
+      <c r="H20" s="1">
+        <v>1</v>
+      </c>
+      <c r="I20" s="1">
+        <v>0.99960259637037996</v>
+      </c>
+      <c r="J20" s="1">
+        <v>0.99973506424692005</v>
+      </c>
+      <c r="K20" s="1">
+        <v>0.99323578133627799</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>16</v>
       </c>
-      <c r="B21">
-        <v>0.92632927610506099</v>
-      </c>
-      <c r="C21">
-        <v>0.832324455205811</v>
-      </c>
-      <c r="D21">
-        <v>0.72186700767263401</v>
-      </c>
-      <c r="E21">
-        <v>0.79300291545189505</v>
-      </c>
-      <c r="F21">
-        <v>0.821710127349909</v>
-      </c>
-      <c r="G21">
-        <v>0.93023255813953498</v>
-      </c>
-      <c r="H21">
-        <v>0.98031496062992196</v>
-      </c>
-      <c r="I21">
-        <v>0.96088019559902305</v>
-      </c>
-      <c r="J21">
-        <v>0.99201596806387304</v>
-      </c>
-      <c r="K21">
-        <v>0.876044568245125</v>
+      <c r="B21" s="1">
+        <v>0.93103448275862</v>
+      </c>
+      <c r="C21" s="1">
+        <v>0.87401574803149595</v>
+      </c>
+      <c r="D21" s="1">
+        <v>0.78008752735229803</v>
+      </c>
+      <c r="E21" s="1">
+        <v>0.81463414634146303</v>
+      </c>
+      <c r="F21" s="1">
+        <v>0.85848074921956297</v>
+      </c>
+      <c r="G21" s="1">
+        <v>0.90500000000000003</v>
+      </c>
+      <c r="H21" s="1">
+        <v>1</v>
+      </c>
+      <c r="I21" s="1">
+        <v>0.99401197604790403</v>
+      </c>
+      <c r="J21" s="1">
+        <v>0.99601593625498097</v>
+      </c>
+      <c r="K21" s="1">
+        <v>0.93874999999999997</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>17</v>
       </c>
-      <c r="B22">
-        <v>0.98499610288386596</v>
-      </c>
-      <c r="C22">
-        <v>0.979848618893149</v>
-      </c>
-      <c r="D22">
-        <v>0.95409804112659602</v>
-      </c>
-      <c r="E22">
-        <v>0.97705242334322495</v>
-      </c>
-      <c r="F22">
-        <v>0.97592374213836497</v>
-      </c>
-      <c r="G22">
-        <v>0.98949109662352797</v>
-      </c>
-      <c r="H22">
-        <v>0.99982327471944898</v>
-      </c>
-      <c r="I22">
-        <v>0.99062718990889997</v>
-      </c>
-      <c r="J22">
-        <v>0.99973507594489597</v>
-      </c>
-      <c r="K22">
-        <v>0.98415413703070098</v>
+      <c r="B22" s="1">
+        <v>0.985194585448393</v>
+      </c>
+      <c r="C22" s="1">
+        <v>0.98673184357541899</v>
+      </c>
+      <c r="D22" s="1">
+        <v>0.96089698668535395</v>
+      </c>
+      <c r="E22" s="1">
+        <v>0.97935649202733499</v>
+      </c>
+      <c r="F22" s="1">
+        <v>0.98095372460496599</v>
+      </c>
+      <c r="G22" s="1">
+        <v>0.99446730032628705</v>
+      </c>
+      <c r="H22" s="1">
+        <v>1</v>
+      </c>
+      <c r="I22" s="1">
+        <v>0.99973502914679402</v>
+      </c>
+      <c r="J22" s="1">
+        <v>1</v>
+      </c>
+      <c r="K22" s="1">
+        <v>0.99255069664781403</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
version up to Chapter 9
</commit_message>
<xml_diff>
--- a/model_comparison.xlsx
+++ b/model_comparison.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gilbertocamara/sitsbook/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63C56649-7722-E14A-81D8-FCC10B584CD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F91FA867-57CD-E84C-BFC4-F52E5B563E01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="30540" windowHeight="18520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-33680" yWindow="-240" windowWidth="23780" windowHeight="14960" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="rfor" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,17 @@
     <sheet name="TempCNN" sheetId="3" r:id="rId3"/>
     <sheet name="LightTAE" sheetId="4" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -84,7 +94,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="168" formatCode="0.000"/>
+    <numFmt numFmtId="164" formatCode="0.000"/>
   </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
@@ -117,7 +127,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1606,6 +1616,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:K22"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="15.5" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A1" t="s">

</xml_diff>